<commit_message>
fix mdms data for commonUiConfig.PrivacyPolicy schema
</commit_message>
<xml_diff>
--- a/jupyter/dataloader/templates/mdms_data.xlsx
+++ b/jupyter/dataloader/templates/mdms_data.xlsx
@@ -1770,406 +1770,406 @@
     <t xml:space="preserve">{"id":"b01cb9ee-1cf6-4b12-990d-a412750088ja","tenantId":"st","schemaCode":"DataSecurity.DecryptionABAC","uniqueIdentifier":"ALL_ACCESS","data":{"key":"ALL_ACCESS","roleAttributeAccessList":[{"roleCode":"CITIZEN","attributeAccessList":[{"attribute":{"jsonPath":"*/name"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/mobileNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/emailId"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/username"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/altContactNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/pan"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/aadhaarNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/guardian"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/permanentAddress/address"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/correspondenceAddress/address"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/addresses/*/address"},"accessType":"PLAIN"}]},{"roleCode":"ANONYMOUS","attributeAccessList":[{"attribute":{"jsonPath":"*/name"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/mobileNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/emailId"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/username"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/altContactNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/pan"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/aadhaarNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/guardian"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/permanentAddress/address"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/correspondenceAddress/address"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/addresses/*/address"},"accessType":"PLAIN"}]},{"roleCode":"EMPLOYEE","attributeAccessList":[{"attribute":{"jsonPath":"*/name"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/mobileNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/emailId"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/username"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/altContactNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/pan"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/aadhaarNumber"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/guardian"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/permanentAddress/address"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/correspondenceAddress/address"},"accessType":"PLAIN"},{"attribute":{"jsonPath":"*/addresses/*/address"},"accessType":"PLAIN"}]}]},"isActive":true,"auditDetails":{"createdBy":"0da6b089-265e-44ef-bf7f-9e0d3ef47bf9","lastModifiedBy":"0da6b089-265e-44ef-bf7f-9e0d3ef47bf9","createdTime":1700804076399,"lastModifiedTime":1700804076399}}</t>
   </si>
   <si>
-    <t xml:space="preserve">  {
-                                        "text": "PRIVACY_HEADER_9_SUB_9_DESC_5_SUBDESC_2",
-                                        "type": "null",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    }
-                                ]
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_10_SUB_10",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_10_SUB_10_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_10_SUB_10_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_11_SUB_11",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_11_SUB_11_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_12_SUB_12",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_12_SUB_12_DESC_1",
-                                "type": "step",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_12_SUB_12_DESC_2",
-                                "type": "step",
-                                "isBold": false
-                            }
-                        ]
-                    }
-                ]
-            },
-            "isActive": true,
-            "auditDetails": {
-                "createdBy": "71d23f7e-30c9-4ba4-b81b-e1862cd3fd9d",
-                "lastModifiedBy": "8a32a4ea-dc0b-465d-b45a-95577475b45d",
-                "createdTime": 1757140063529,
-                "lastModifiedTime": 1766381031261
-            }
-        }
-            "id": "da30d4ad-2111-48f4-8539-03e81f706069",
-            "tenantId": "st",
-            "schemaCode": "commonUiConfig.PrivacyPolicy",
-            "uniqueIdentifier": "HCM",
-            "data": {
-                "header": "PRIVACY_HEADER",
-                "module": "HCM",
-                "contents": [
-                    {
-                        "header": "PRIVACY_HEADER_1_SUB_1",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_1_SUB_1_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_1_SUB_1_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_1_SUB_1_DESC_3",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_1_SUB_1_DESC_4",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_1_SUB_1_DESC_5",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_1_SUB_1_DESC_6",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_1_SUB_1_DESC_7",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_2_SUB_2",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_2_SUB_2_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_2_SUB_2_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_2_SUB_2_DESC_3",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_2_SUB_2_DESC_4",
-                                "type": "null",
-                                "isBold": false,
-                                "subDescriptions": [
-                                    {
-                                        "text": "PRIVACY_HEADER_2_SUB_2_DESC_3_SUBDESC_1",
-                                        "type": "null",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_2_SUB_2_DESC_3_SUBDESC_2",
-                                        "type": "null",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    }
-                                ]
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_2_SUB_2_DESC_5",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_3_SUB_3",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_3_SUB_3_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_3_SUB_3_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_4_SUB_4",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_4_SUB_4_DESC_1",
-                                "type": "null",
-                                "isBold": false,
-                                "subDescriptions": [
-                                    {
-                                        "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_1",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_2",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_3",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_4",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_5",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_6",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_7",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    }
-                                ]
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_4_SUB_4_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_5_SUB_5",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_5_SUB_5_DESC_1",
-                                "type": "null",
-                                "isBold": false,
-                                "subDescriptions": [
-                                    {
-                                        "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_1",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_2",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_3",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_4",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_5",
-                                        "type": "points",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    }
-                                ]
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_6_SUB_1",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_6_SUB_6_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_6_SUB_6_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_6_SUB_6_DESC_3",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_6_SUB_6_DESC_4",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_7_SUB_1",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_7_SUB_7_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_7_SUB_7_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_7_SUB_7_DESC_3",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_7_SUB_7_DESC_4",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_8_SUB_1",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_8_SUB_8_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_8_SUB_8_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_8_SUB_8_DESC_3",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_8_SUB_8_DESC_4",
-                                "type": "null",
-                                "isBold": false
-                            }
-                        ]
-                    },
-                    {
-                        "header": "PRIVACY_HEADER_9_SUB_9",
-                        "descriptions": [
-                            {
-                                "text": "PRIVACY_HEADER_9_SUB_9_DESC_1",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_9_SUB_9_DESC_2",
-                                "type": "null",
-                                "isBold": false
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_9_SUB_9_DESC_3",
-                                "type": "null",
-                                "isBold": false,
-                                "subDescriptions": [
-                                    {
-                                        "text": "PRIVACY_HEADER_9_SUB_9_DESC_3_SUBDESC_1",
-                                        "type": "null",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {
-                                        "text": "PRIVACY_HEADER_9_SUB_9_DESC_3_SUBDESC_2",
-                                        "type": "null",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    }
-                                ]
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_9_SUB_9_DESC_4",
-                                "type": "null",
-                                "isBold": false,
-                                "subDescriptions": [
-                                    {
-                                        "text": "PRIVACY_HEADER_9_SUB_9_DESC_4_SUBDESC_1",
-                                        "type": "null",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    }
-                                ]
-                            },
-                            {
-                                "text": "PRIVACY_HEADER_9_SUB_9_DESC_5",
-                                "type": "null",
-                                "isBold": false,
-                                "subDescriptions": [
-                                    {
-                                        "text": "PRIVACY_HEADER_9_SUB_9_DESC_5_SUBDESC_1",
-                                        "type": "null",
-                                        "isBold": false,
-                                        "isSpaceRequired": true
-                                    },
-                                    {</t>
+    <t xml:space="preserve">{
+  "id": "da30d4ad-2111-48f4-8539-03e81f706069",
+  "tenantId": "st",
+  "schemaCode": "commonUiConfig.PrivacyPolicy",
+  "uniqueIdentifier": "HCM",
+  "data": {
+    "header": "PRIVACY_HEADER",
+    "module": "HCM",
+    "contents": [
+      {
+        "header": "PRIVACY_HEADER_1_SUB_1",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_1_SUB_1_DESC_1",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_1_SUB_1_DESC_2",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_1_SUB_1_DESC_3",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_1_SUB_1_DESC_4",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_1_SUB_1_DESC_5",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_1_SUB_1_DESC_6",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_1_SUB_1_DESC_7",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_2_SUB_2",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_2_SUB_2_DESC_1",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_2_SUB_2_DESC_2",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_2_SUB_2_DESC_3",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_2_SUB_2_DESC_4",
+            "type": "null",
+            "isBold": false,
+            "subDescriptions": [
+              {
+                "text": "PRIVACY_HEADER_2_SUB_2_DESC_3_SUBDESC_1",
+                "type": "null",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_2_SUB_2_DESC_3_SUBDESC_2",
+                "type": "null",
+                "isBold": false,
+                "isSpaceRequired": true
+              }
+            ]
+          },
+          {
+            "text": "PRIVACY_HEADER_2_SUB_2_DESC_5",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_3_SUB_3",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_3_SUB_3_DESC_1",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_3_SUB_3_DESC_2",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_4_SUB_4",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_4_SUB_4_DESC_1",
+            "type": "null",
+            "isBold": false,
+            "subDescriptions": [
+              {
+                "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_1",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_2",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_3",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_4",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_5",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_6",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_4_SUB_4_DESC_1_SUBDESC_7",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              }
+            ]
+          },
+          {
+            "text": "PRIVACY_HEADER_4_SUB_4_DESC_2",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_5_SUB_5",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_5_SUB_5_DESC_1",
+            "type": "null",
+            "isBold": false,
+            "subDescriptions": [
+              {
+                "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_1",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_2",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_3",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_4",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_5_SUB_5_DESC_1_SUBDESC_5",
+                "type": "points",
+                "isBold": false,
+                "isSpaceRequired": true
+              }
+            ]
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_6_SUB_1",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_6_SUB_6_DESC_1",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_6_SUB_6_DESC_2",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_6_SUB_6_DESC_3",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_6_SUB_6_DESC_4",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_7_SUB_1",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_7_SUB_7_DESC_1",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_7_SUB_7_DESC_2",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_7_SUB_7_DESC_3",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_7_SUB_7_DESC_4",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_8_SUB_1",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_8_SUB_8_DESC_1",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_8_SUB_8_DESC_2",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_8_SUB_8_DESC_3",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_8_SUB_8_DESC_4",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_9_SUB_9",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_9_SUB_9_DESC_1",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_9_SUB_9_DESC_2",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_9_SUB_9_DESC_3",
+            "type": "null",
+            "isBold": false,
+            "subDescriptions": [
+              {
+                "text": "PRIVACY_HEADER_9_SUB_9_DESC_3_SUBDESC_1",
+                "type": "null",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_9_SUB_9_DESC_3_SUBDESC_2",
+                "type": "null",
+                "isBold": false,
+                "isSpaceRequired": true
+              }
+            ]
+          },
+          {
+            "text": "PRIVACY_HEADER_9_SUB_9_DESC_4",
+            "type": "null",
+            "isBold": false,
+            "subDescriptions": [
+              {
+                "text": "PRIVACY_HEADER_9_SUB_9_DESC_4_SUBDESC_1",
+                "type": "null",
+                "isBold": false,
+                "isSpaceRequired": true
+              }
+            ]
+          },
+          {
+            "text": "PRIVACY_HEADER_9_SUB_9_DESC_5",
+            "type": "null",
+            "isBold": false,
+            "subDescriptions": [
+              {
+                "text": "PRIVACY_HEADER_9_SUB_9_DESC_5_SUBDESC_1",
+                "type": "null",
+                "isBold": false,
+                "isSpaceRequired": true
+              },
+              {
+                "text": "PRIVACY_HEADER_9_SUB_9_DESC_5_SUBDESC_2",
+                "type": "null",
+                "isBold": false,
+                "isSpaceRequired": true
+              }
+            ]
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_10_SUB_10",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_10_SUB_10_DESC_1",
+            "type": "null",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_10_SUB_10_DESC_2",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_11_SUB_11",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_11_SUB_11_DESC_1",
+            "type": "null",
+            "isBold": false
+          }
+        ]
+      },
+      {
+        "header": "PRIVACY_HEADER_12_SUB_12",
+        "descriptions": [
+          {
+            "text": "PRIVACY_HEADER_12_SUB_12_DESC_1",
+            "type": "step",
+            "isBold": false
+          },
+          {
+            "text": "PRIVACY_HEADER_12_SUB_12_DESC_2",
+            "type": "step",
+            "isBold": false
+          }
+        ]
+      }
+    ]
+  },
+  "isActive": true,
+  "auditDetails": {
+    "createdBy": "71d23f7e-30c9-4ba4-b81b-e1862cd3fd9d",
+    "lastModifiedBy": "8a32a4ea-dc0b-465d-b45a-95577475b45d",
+    "createdTime": 1757140063529,
+    "lastModifiedTime": 1766381031261
+  }
+}</t>
   </si>
   <si>
     <t xml:space="preserve">  {
@@ -4165,6 +4165,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -4186,18 +4187,21 @@
       <color rgb="FF000000"/>
       <name val="'Droid Sans Mono'"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Droid Sans Mono"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <u val="single"/>
@@ -4205,24 +4209,28 @@
       <color rgb="FF0000FF"/>
       <name val="Cambria"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF1D1C1D"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Monaco"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="&quot;Inter Variable&quot;"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -8713,14 +8721,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z1048576"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Z247"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="72" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="116.13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
         <v>86</v>
       </c>
@@ -8728,7 +8736,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -8736,7 +8744,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="470.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
@@ -8744,7 +8752,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
@@ -8752,7 +8760,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>20</v>
       </c>
@@ -8760,7 +8768,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
@@ -8768,7 +8776,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>20</v>
       </c>
@@ -8776,7 +8784,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
         <v>20</v>
       </c>
@@ -8784,7 +8792,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
         <v>20</v>
       </c>
@@ -8792,7 +8800,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>20</v>
       </c>
@@ -8800,7 +8808,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
@@ -8808,7 +8816,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
         <v>20</v>
       </c>
@@ -8816,7 +8824,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
         <v>20</v>
       </c>
@@ -8824,7 +8832,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
         <v>22</v>
       </c>
@@ -8832,7 +8840,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
         <v>22</v>
       </c>
@@ -8840,7 +8848,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
         <v>22</v>
       </c>
@@ -8848,7 +8856,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
         <v>22</v>
       </c>
@@ -8856,7 +8864,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
         <v>22</v>
       </c>
@@ -8864,7 +8872,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
@@ -8872,7 +8880,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>22</v>
       </c>
@@ -8880,7 +8888,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
         <v>22</v>
       </c>
@@ -8888,7 +8896,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
         <v>22</v>
       </c>
@@ -8896,7 +8904,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
         <v>22</v>
       </c>
@@ -8904,7 +8912,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
         <v>22</v>
       </c>
@@ -8912,7 +8920,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
         <v>22</v>
       </c>
@@ -8920,7 +8928,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
         <v>22</v>
       </c>
@@ -8928,7 +8936,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>22</v>
       </c>
@@ -8936,7 +8944,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
         <v>26</v>
       </c>
@@ -8944,7 +8952,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
@@ -8952,7 +8960,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
         <v>30</v>
       </c>
@@ -8960,7 +8968,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
         <v>30</v>
       </c>
@@ -8968,7 +8976,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="222.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
         <v>32</v>
       </c>
@@ -8976,7 +8984,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
         <v>119</v>
       </c>
@@ -8984,7 +8992,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
         <v>119</v>
       </c>
@@ -8992,7 +9000,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
         <v>119</v>
       </c>
@@ -9000,7 +9008,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
         <v>36</v>
       </c>
@@ -9008,7 +9016,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
         <v>36</v>
       </c>
@@ -9016,7 +9024,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
         <v>36</v>
       </c>
@@ -9024,7 +9032,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
         <v>36</v>
       </c>
@@ -9032,7 +9040,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
         <v>36</v>
       </c>
@@ -9040,7 +9048,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
         <v>36</v>
       </c>
@@ -9048,7 +9056,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
         <v>38</v>
       </c>
@@ -9056,7 +9064,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
         <v>38</v>
       </c>
@@ -9064,7 +9072,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
         <v>40</v>
       </c>
@@ -9072,7 +9080,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
         <v>40</v>
       </c>
@@ -9080,7 +9088,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
         <v>40</v>
       </c>
@@ -9088,7 +9096,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
         <v>40</v>
       </c>
@@ -9096,7 +9104,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
         <v>40</v>
       </c>
@@ -9104,7 +9112,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
         <v>40</v>
       </c>
@@ -9112,7 +9120,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
         <v>40</v>
       </c>
@@ -9120,7 +9128,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
         <v>40</v>
       </c>
@@ -9128,7 +9136,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
         <v>40</v>
       </c>
@@ -9136,7 +9144,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
         <v>40</v>
       </c>
@@ -9144,7 +9152,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
         <v>42</v>
       </c>
@@ -9152,7 +9160,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
         <v>42</v>
       </c>
@@ -9160,7 +9168,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="318.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
         <v>44</v>
       </c>
@@ -9168,7 +9176,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="458.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
         <v>44</v>
       </c>
@@ -9176,7 +9184,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="686.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
         <v>44</v>
       </c>
@@ -9184,7 +9192,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
         <v>44</v>
       </c>
@@ -9192,7 +9200,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="305.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="s">
         <v>46</v>
       </c>
@@ -9200,7 +9208,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
         <v>48</v>
       </c>
@@ -9208,7 +9216,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="305.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
         <v>48</v>
       </c>
@@ -9216,7 +9224,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
         <v>50</v>
       </c>
@@ -9224,7 +9232,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
         <v>50</v>
       </c>
@@ -9232,7 +9240,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="6" t="s">
         <v>50</v>
       </c>
@@ -9240,7 +9248,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="s">
         <v>50</v>
       </c>
@@ -9248,7 +9256,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="s">
         <v>50</v>
       </c>
@@ -9256,7 +9264,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="6" t="s">
         <v>50</v>
       </c>
@@ -9264,7 +9272,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
         <v>52</v>
       </c>
@@ -9272,7 +9280,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="s">
         <v>52</v>
       </c>
@@ -9280,7 +9288,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="s">
         <v>52</v>
       </c>
@@ -9288,7 +9296,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="s">
         <v>52</v>
       </c>
@@ -9296,7 +9304,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="s">
         <v>52</v>
       </c>
@@ -9304,7 +9312,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
         <v>52</v>
       </c>
@@ -9312,7 +9320,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
         <v>52</v>
       </c>
@@ -9320,7 +9328,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="s">
         <v>52</v>
       </c>
@@ -9328,7 +9336,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="534.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
         <v>54</v>
       </c>
@@ -9336,7 +9344,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="788.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
         <v>54</v>
       </c>
@@ -9344,7 +9352,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="s">
         <v>56</v>
       </c>
@@ -9352,7 +9360,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="s">
         <v>56</v>
       </c>
@@ -9360,7 +9368,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="6" t="s">
         <v>56</v>
       </c>
@@ -9368,7 +9376,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="6" t="s">
         <v>56</v>
       </c>
@@ -9376,7 +9384,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="6" t="s">
         <v>56</v>
       </c>
@@ -9384,7 +9392,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="6" t="s">
         <v>56</v>
       </c>
@@ -9392,7 +9400,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="6" t="s">
         <v>56</v>
       </c>
@@ -9400,7 +9408,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="6" t="s">
         <v>56</v>
       </c>
@@ -9408,7 +9416,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="6" t="s">
         <v>56</v>
       </c>
@@ -9416,7 +9424,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="6" t="s">
         <v>56</v>
       </c>
@@ -9424,7 +9432,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="6" t="s">
         <v>56</v>
       </c>
@@ -9432,7 +9440,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="6" t="s">
         <v>56</v>
       </c>
@@ -9440,7 +9448,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="6" t="s">
         <v>56</v>
       </c>
@@ -9448,7 +9456,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="6" t="s">
         <v>56</v>
       </c>
@@ -9456,7 +9464,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="1053.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="6" t="s">
         <v>58</v>
       </c>
@@ -9464,7 +9472,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="1131.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="6" t="s">
         <v>60</v>
       </c>
@@ -9472,7 +9480,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="1296.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="6" t="s">
         <v>62</v>
       </c>
@@ -9480,7 +9488,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="559.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="6" t="s">
         <v>183</v>
       </c>
@@ -9488,7 +9496,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="1765.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="6" t="s">
         <v>183</v>
       </c>
@@ -9496,7 +9504,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="1473.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="6" t="s">
         <v>64</v>
       </c>
@@ -9504,7 +9512,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="6" t="s">
         <v>68</v>
       </c>
@@ -9512,7 +9520,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="6" t="s">
         <v>68</v>
       </c>
@@ -9520,7 +9528,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="6" t="s">
         <v>68</v>
       </c>
@@ -9528,7 +9536,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="6" t="s">
         <v>70</v>
       </c>
@@ -9536,7 +9544,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="6" t="s">
         <v>70</v>
       </c>
@@ -9544,7 +9552,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="6" t="s">
         <v>70</v>
       </c>
@@ -9552,7 +9560,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="6" t="s">
         <v>70</v>
       </c>
@@ -9560,7 +9568,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="6" t="s">
         <v>70</v>
       </c>
@@ -9568,7 +9576,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="6" t="s">
         <v>70</v>
       </c>
@@ -9576,7 +9584,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="6" t="s">
         <v>70</v>
       </c>
@@ -9584,7 +9592,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="6" t="s">
         <v>70</v>
       </c>
@@ -9592,7 +9600,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="6" t="s">
         <v>70</v>
       </c>
@@ -9600,7 +9608,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="6" t="s">
         <v>70</v>
       </c>
@@ -9608,7 +9616,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="6" t="s">
         <v>70</v>
       </c>
@@ -9616,7 +9624,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="6" t="s">
         <v>70</v>
       </c>
@@ -9624,7 +9632,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="6" t="s">
         <v>70</v>
       </c>
@@ -9632,7 +9640,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="6" t="s">
         <v>70</v>
       </c>
@@ -9640,7 +9648,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="6" t="s">
         <v>70</v>
       </c>
@@ -9648,7 +9656,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="6" t="s">
         <v>70</v>
       </c>
@@ -9656,7 +9664,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="6" t="s">
         <v>70</v>
       </c>
@@ -9664,7 +9672,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="6" t="s">
         <v>70</v>
       </c>
@@ -9672,7 +9680,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="6" t="s">
         <v>70</v>
       </c>
@@ -9680,7 +9688,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="6" t="s">
         <v>70</v>
       </c>
@@ -9688,7 +9696,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="6" t="s">
         <v>70</v>
       </c>
@@ -9696,7 +9704,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="6" t="s">
         <v>70</v>
       </c>
@@ -9704,7 +9712,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="6" t="s">
         <v>70</v>
       </c>
@@ -9712,7 +9720,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="6" t="s">
         <v>70</v>
       </c>
@@ -9720,7 +9728,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="6" t="s">
         <v>70</v>
       </c>
@@ -9728,7 +9736,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="6" t="s">
         <v>70</v>
       </c>
@@ -9736,7 +9744,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="6" t="s">
         <v>70</v>
       </c>
@@ -9744,7 +9752,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="6" t="s">
         <v>70</v>
       </c>
@@ -9752,7 +9760,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="6" t="s">
         <v>70</v>
       </c>
@@ -9760,7 +9768,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="242.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="6" t="s">
         <v>72</v>
       </c>
@@ -9768,7 +9776,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="242.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="6" t="s">
         <v>72</v>
       </c>
@@ -9776,7 +9784,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="242.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="6" t="s">
         <v>72</v>
       </c>
@@ -9784,7 +9792,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="6" t="s">
         <v>72</v>
       </c>
@@ -9792,7 +9800,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="6" t="s">
         <v>72</v>
       </c>
@@ -9800,7 +9808,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="6" t="s">
         <v>72</v>
       </c>
@@ -9808,7 +9816,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="6" t="s">
         <v>72</v>
       </c>
@@ -9816,7 +9824,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="6" t="s">
         <v>72</v>
       </c>
@@ -9824,7 +9832,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="6" t="s">
         <v>72</v>
       </c>
@@ -9832,7 +9840,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="6" t="s">
         <v>72</v>
       </c>
@@ -9840,7 +9848,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="6" t="s">
         <v>72</v>
       </c>
@@ -9848,7 +9856,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="6" t="s">
         <v>72</v>
       </c>
@@ -9856,7 +9864,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="6" t="s">
         <v>72</v>
       </c>
@@ -9864,7 +9872,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="6" t="s">
         <v>72</v>
       </c>
@@ -9872,7 +9880,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="6" t="s">
         <v>72</v>
       </c>
@@ -9880,7 +9888,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="6" t="s">
         <v>72</v>
       </c>
@@ -9888,7 +9896,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="6" t="s">
         <v>72</v>
       </c>
@@ -9896,7 +9904,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="267.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="6" t="s">
         <v>236</v>
       </c>
@@ -9904,7 +9912,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="267.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="6" t="s">
         <v>236</v>
       </c>
@@ -9912,7 +9920,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="293.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="6" t="s">
         <v>239</v>
       </c>
@@ -9920,7 +9928,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="293.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="6" t="s">
         <v>239</v>
       </c>
@@ -9928,7 +9936,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="356.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="6" t="s">
         <v>242</v>
       </c>
@@ -9936,7 +9944,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="356.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="6" t="s">
         <v>242</v>
       </c>
@@ -9944,7 +9952,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="547" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="6" t="s">
         <v>82</v>
       </c>
@@ -9952,7 +9960,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="6" t="s">
         <v>84</v>
       </c>
@@ -9960,7 +9968,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="6" t="s">
         <v>84</v>
       </c>
@@ -9968,7 +9976,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="6" t="s">
         <v>84</v>
       </c>
@@ -9976,7 +9984,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="6" t="s">
         <v>84</v>
       </c>
@@ -9984,7 +9992,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="6" t="s">
         <v>84</v>
       </c>
@@ -9992,7 +10000,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="6" t="s">
         <v>84</v>
       </c>
@@ -10000,7 +10008,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="6" t="s">
         <v>84</v>
       </c>
@@ -10008,7 +10016,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="6" t="s">
         <v>84</v>
       </c>
@@ -10016,7 +10024,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="6" t="s">
         <v>84</v>
       </c>
@@ -10024,7 +10032,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="6" t="s">
         <v>84</v>
       </c>
@@ -10032,7 +10040,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="6" t="s">
         <v>84</v>
       </c>
@@ -10040,7 +10048,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="6" t="s">
         <v>84</v>
       </c>
@@ -10048,7 +10056,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="6" t="s">
         <v>84</v>
       </c>
@@ -10056,7 +10064,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="6" t="s">
         <v>84</v>
       </c>
@@ -10064,7 +10072,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="6" t="s">
         <v>80</v>
       </c>
@@ -10072,7 +10080,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="6" t="s">
         <v>80</v>
       </c>
@@ -10080,7 +10088,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="6" t="s">
         <v>80</v>
       </c>
@@ -10088,7 +10096,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="6" t="s">
         <v>80</v>
       </c>
@@ -10096,7 +10104,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="6" t="s">
         <v>80</v>
       </c>
@@ -10128,7 +10136,7 @@
       <c r="Y173" s="7"/>
       <c r="Z173" s="7"/>
     </row>
-    <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="6" t="s">
         <v>80</v>
       </c>
@@ -10160,7 +10168,7 @@
       <c r="Y174" s="7"/>
       <c r="Z174" s="7"/>
     </row>
-    <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="6" t="s">
         <v>80</v>
       </c>
@@ -10192,7 +10200,7 @@
       <c r="Y175" s="7"/>
       <c r="Z175" s="7"/>
     </row>
-    <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="6" t="s">
         <v>80</v>
       </c>
@@ -10224,7 +10232,7 @@
       <c r="Y176" s="7"/>
       <c r="Z176" s="7"/>
     </row>
-    <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="6" t="s">
         <v>80</v>
       </c>
@@ -10232,7 +10240,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="6" t="s">
         <v>80</v>
       </c>
@@ -10240,7 +10248,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="6" t="s">
         <v>80</v>
       </c>
@@ -10272,7 +10280,7 @@
       <c r="Y179" s="7"/>
       <c r="Z179" s="7"/>
     </row>
-    <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="6" t="s">
         <v>80</v>
       </c>
@@ -10280,7 +10288,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="6" t="s">
         <v>80</v>
       </c>
@@ -10288,7 +10296,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="6" t="s">
         <v>80</v>
       </c>
@@ -10320,7 +10328,7 @@
       <c r="Y182" s="7"/>
       <c r="Z182" s="7"/>
     </row>
-    <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="6" t="s">
         <v>80</v>
       </c>
@@ -10352,7 +10360,7 @@
       <c r="Y183" s="7"/>
       <c r="Z183" s="7"/>
     </row>
-    <row r="184" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="6" t="s">
         <v>74</v>
       </c>
@@ -10360,7 +10368,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="6" t="s">
         <v>74</v>
       </c>
@@ -10368,7 +10376,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="6" t="s">
         <v>74</v>
       </c>
@@ -10376,7 +10384,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="6" t="s">
         <v>74</v>
       </c>
@@ -10384,7 +10392,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="6" t="s">
         <v>74</v>
       </c>
@@ -10392,7 +10400,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="6" t="s">
         <v>74</v>
       </c>
@@ -10400,7 +10408,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="190" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="6" t="s">
         <v>74</v>
       </c>
@@ -10408,7 +10416,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="6" t="s">
         <v>76</v>
       </c>
@@ -10416,7 +10424,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="6" t="s">
         <v>76</v>
       </c>
@@ -10424,7 +10432,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="6" t="s">
         <v>76</v>
       </c>
@@ -10432,7 +10440,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="6" t="s">
         <v>76</v>
       </c>
@@ -10440,7 +10448,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="6" t="s">
         <v>76</v>
       </c>
@@ -10448,7 +10456,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="6" t="s">
         <v>76</v>
       </c>
@@ -10456,7 +10464,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="6" t="s">
         <v>76</v>
       </c>
@@ -10464,7 +10472,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="6" t="s">
         <v>76</v>
       </c>
@@ -10472,7 +10480,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="6" t="s">
         <v>76</v>
       </c>
@@ -10480,7 +10488,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="6" t="s">
         <v>76</v>
       </c>
@@ -10488,7 +10496,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="6" t="s">
         <v>76</v>
       </c>
@@ -10496,7 +10504,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="6" t="s">
         <v>76</v>
       </c>
@@ -10504,7 +10512,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="6" t="s">
         <v>76</v>
       </c>
@@ -10512,7 +10520,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="6" t="s">
         <v>76</v>
       </c>
@@ -10520,7 +10528,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="6" t="s">
         <v>76</v>
       </c>
@@ -10528,7 +10536,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="6" t="s">
         <v>76</v>
       </c>
@@ -10536,7 +10544,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="6" t="s">
         <v>76</v>
       </c>
@@ -10544,7 +10552,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="6" t="s">
         <v>76</v>
       </c>
@@ -10552,7 +10560,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="6" t="s">
         <v>76</v>
       </c>
@@ -10560,7 +10568,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="6" t="s">
         <v>76</v>
       </c>
@@ -10568,7 +10576,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="6" t="s">
         <v>78</v>
       </c>
@@ -10576,7 +10584,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="6" t="s">
         <v>78</v>
       </c>
@@ -10584,7 +10592,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="6" t="s">
         <v>78</v>
       </c>
@@ -10592,7 +10600,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="6" t="s">
         <v>78</v>
       </c>
@@ -10600,7 +10608,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="6" t="s">
         <v>78</v>
       </c>
@@ -10608,7 +10616,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="6" t="s">
         <v>78</v>
       </c>
@@ -10616,7 +10624,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="6" t="s">
         <v>78</v>
       </c>
@@ -10624,7 +10632,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="6" t="s">
         <v>78</v>
       </c>
@@ -10632,7 +10640,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="6" t="s">
         <v>78</v>
       </c>
@@ -10640,7 +10648,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="6" t="s">
         <v>78</v>
       </c>
@@ -10648,7 +10656,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="6" t="s">
         <v>78</v>
       </c>
@@ -10656,7 +10664,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="6" t="s">
         <v>78</v>
       </c>
@@ -10664,7 +10672,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A223" s="6" t="s">
         <v>78</v>
       </c>
@@ -10672,7 +10680,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="6" t="s">
         <v>78</v>
       </c>
@@ -10680,7 +10688,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A225" s="6" t="s">
         <v>78</v>
       </c>
@@ -10688,7 +10696,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="6" t="s">
         <v>78</v>
       </c>
@@ -10696,7 +10704,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A227" s="6" t="s">
         <v>78</v>
       </c>
@@ -10704,7 +10712,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A228" s="6" t="s">
         <v>78</v>
       </c>
@@ -10712,7 +10720,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A229" s="6" t="s">
         <v>78</v>
       </c>
@@ -10720,7 +10728,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A230" s="6" t="s">
         <v>78</v>
       </c>
@@ -10728,7 +10736,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A231" s="6" t="s">
         <v>78</v>
       </c>
@@ -10736,7 +10744,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="232" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A232" s="6" t="s">
         <v>78</v>
       </c>
@@ -10744,7 +10752,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="233" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="233" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="6" t="s">
         <v>78</v>
       </c>
@@ -10752,7 +10760,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="6" t="s">
         <v>78</v>
       </c>
@@ -10760,7 +10768,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="6" t="s">
         <v>78</v>
       </c>
@@ -10768,7 +10776,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A236" s="6" t="s">
         <v>78</v>
       </c>
@@ -10776,7 +10784,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A237" s="6" t="s">
         <v>78</v>
       </c>
@@ -10784,7 +10792,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="238" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="238" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A238" s="6" t="s">
         <v>78</v>
       </c>
@@ -10792,7 +10800,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="239" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="239" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A239" s="6" t="s">
         <v>78</v>
       </c>
@@ -10800,7 +10808,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A240" s="6" t="s">
         <v>78</v>
       </c>
@@ -10808,7 +10816,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A241" s="6" t="s">
         <v>78</v>
       </c>
@@ -10816,7 +10824,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A242" s="6" t="s">
         <v>78</v>
       </c>
@@ -10824,7 +10832,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="243" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A243" s="6" t="s">
         <v>78</v>
       </c>
@@ -10832,7 +10840,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="244" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="244" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A244" s="6" t="s">
         <v>78</v>
       </c>
@@ -10840,7 +10848,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A245" s="6" t="s">
         <v>78</v>
       </c>
@@ -10848,7 +10856,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="246" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A246" s="6" t="s">
         <v>78</v>
       </c>
@@ -10856,7 +10864,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="247" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="247" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A247" s="6" t="s">
         <v>78</v>
       </c>
@@ -10864,18 +10872,6 @@
         <v>337</v>
       </c>
     </row>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
@@ -10918,77 +10914,77 @@
         <v>341</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3"/>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3"/>
     </row>
-    <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3"/>
     </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3"/>
     </row>
-    <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
         <v>353</v>
       </c>
@@ -10998,7 +10994,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>355</v>
       </c>
@@ -14016,7 +14012,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>
       <c r="B12" s="3" t="s">
         <v>367</v>
@@ -14132,7 +14128,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14"/>
       <c r="B30" s="3" t="s">
         <v>385</v>
@@ -14154,13 +14150,13 @@
         <v>387</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14"/>
       <c r="B33" s="3" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14"/>
       <c r="B34" s="3" t="s">
         <v>389</v>
@@ -14174,31 +14170,31 @@
         <v>390</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14"/>
       <c r="B36" s="3" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14"/>
       <c r="B37" s="3" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14"/>
       <c r="B38" s="3" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14"/>
       <c r="B39" s="3" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14"/>
       <c r="B40" s="3" t="s">
         <v>395</v>
@@ -14212,7 +14208,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14"/>
       <c r="B42" s="3" t="s">
         <v>397</v>
@@ -14226,55 +14222,55 @@
         <v>398</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14"/>
       <c r="B44" s="3" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14"/>
       <c r="B45" s="3" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14"/>
       <c r="B46" s="3" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14"/>
       <c r="B47" s="3" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14"/>
       <c r="B48" s="3" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14"/>
       <c r="B49" s="3" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14"/>
       <c r="B50" s="3" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14"/>
       <c r="B51" s="3" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14"/>
       <c r="B52" s="3" t="s">
         <v>407</v>
@@ -14288,7 +14284,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="15"/>
       <c r="B54" s="3" t="s">
         <v>409</v>
@@ -14388,43 +14384,43 @@
         <v>423</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="15"/>
       <c r="B69" s="3" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="15"/>
       <c r="B70" s="3" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="15"/>
       <c r="B71" s="3" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="15"/>
       <c r="B72" s="3" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="15"/>
       <c r="B73" s="3" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="15"/>
       <c r="B74" s="3" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="15"/>
       <c r="B75" s="3" t="s">
         <v>430</v>
@@ -14584,13 +14580,13 @@
         <v>453</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="15"/>
       <c r="B99" s="3" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="15"/>
       <c r="B100" s="3" t="s">
         <v>399</v>
@@ -14604,133 +14600,133 @@
         <v>455</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="15"/>
       <c r="B102" s="3" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="15"/>
       <c r="B103" s="3" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="15"/>
       <c r="B104" s="3" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="15"/>
       <c r="B105" s="3" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="15"/>
       <c r="B106" s="3" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="15"/>
       <c r="B107" s="3" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="15"/>
       <c r="B108" s="3" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="15"/>
       <c r="B109" s="3" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="15"/>
       <c r="B110" s="3" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="15"/>
       <c r="B111" s="3" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="15"/>
       <c r="B112" s="3" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="15"/>
       <c r="B113" s="3" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="15"/>
       <c r="B114" s="3" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="15"/>
       <c r="B115" s="3" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="15"/>
       <c r="B116" s="3" t="s">
         <v>470</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="15"/>
       <c r="B117" s="3" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="15"/>
       <c r="B118" s="3" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="15"/>
       <c r="B119" s="3" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="15"/>
       <c r="B120" s="3" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="15"/>
       <c r="B121" s="3" t="s">
         <v>475</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="15"/>
       <c r="B122" s="3" t="s">
         <v>476</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="15"/>
       <c r="B123" s="3" t="s">
         <v>477</v>
@@ -14742,31 +14738,31 @@
         <v>478</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="15"/>
       <c r="B125" s="3" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="15"/>
       <c r="B126" s="3" t="s">
         <v>480</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="15"/>
       <c r="B127" s="3" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="15"/>
       <c r="B128" s="3" t="s">
         <v>482</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="15"/>
       <c r="B129" s="3" t="s">
         <v>483</v>
@@ -14780,97 +14776,97 @@
         <v>484</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="15"/>
       <c r="B131" s="3" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="15"/>
       <c r="B132" s="3" t="s">
         <v>486</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="15"/>
       <c r="B133" s="3" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="15"/>
       <c r="B134" s="3" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="15"/>
       <c r="B135" s="3" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="15"/>
       <c r="B136" s="3" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="15"/>
       <c r="B137" s="3" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="15"/>
       <c r="B138" s="3" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="15"/>
       <c r="B139" s="3" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="15"/>
       <c r="B140" s="3" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="15"/>
       <c r="B141" s="3" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="15"/>
       <c r="B142" s="3" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="15"/>
       <c r="B143" s="3" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="15"/>
       <c r="B144" s="3" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="15"/>
       <c r="B145" s="3" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="15"/>
       <c r="B146" s="3" t="s">
         <v>500</v>
@@ -14934,79 +14930,79 @@
         <v>508</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="15"/>
       <c r="B155" s="3" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="15"/>
       <c r="B156" s="3" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="15"/>
       <c r="B157" s="3" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="15"/>
       <c r="B158" s="3" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="15"/>
       <c r="B159" s="3" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="15"/>
       <c r="B160" s="3" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="15"/>
       <c r="B161" s="3" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="15"/>
       <c r="B162" s="3" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="15"/>
       <c r="B163" s="3" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="15"/>
       <c r="B164" s="3" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="15"/>
       <c r="B165" s="3" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="15"/>
       <c r="B166" s="3" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="15"/>
       <c r="B167" s="3" t="s">
         <v>520</v>
@@ -15032,7 +15028,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="15"/>
       <c r="B171" s="3" t="s">
         <v>524</v>
@@ -15044,19 +15040,19 @@
         <v>525</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="15"/>
       <c r="B173" s="3" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="15"/>
       <c r="B174" s="3" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="15"/>
       <c r="B175" s="3" t="s">
         <v>528</v>
@@ -15070,7 +15066,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="15"/>
       <c r="B177" s="3" t="s">
         <v>530</v>
@@ -15082,25 +15078,25 @@
         <v>531</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="15"/>
       <c r="B179" s="3" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="15"/>
       <c r="B180" s="3" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="15"/>
       <c r="B181" s="3" t="s">
         <v>534</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="15"/>
       <c r="B182" s="3" t="s">
         <v>535</v>

</xml_diff>